<commit_message>
lab2-3: seven Excel workbooks filled via COM, results json
</commit_message>
<xml_diff>
--- a/ЛР2-3_Объем_рынка/Excel/ЛР2-3_1_потенциальные_клиенты_TableMind.xlsx
+++ b/ЛР2-3_Объем_рынка/Excel/ЛР2-3_1_потенциальные_клиенты_TableMind.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-continuation-3ab569\ЛР2-3_Объем_рынка\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65B9E5A6-16C7-4775-8EDF-49AADB62CD37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ED63552-C1B6-4CDF-B6C1-CFE528702DBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="368" yWindow="368" windowWidth="12022" windowHeight="10972" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -611,9 +611,6 @@
     <t>Шаблон итогового вывода</t>
   </si>
   <si>
-    <t>По результатам оценки через количество потенциальных клиентов базовый доступный объем рынка составляет ориентировочно [SAM] BYN в год, а реалистично достижимый объем для нового бизнеса составляет [SOM] BYN в год. Оценка является сценарной и требует проверки через фактические данные о клиентах, конкурентах, рекламных каналах, Similarweb, поисковом спросе и платежеспособности целевых сегментов.</t>
-  </si>
-  <si>
     <t>Журнал источников данных и допущений</t>
   </si>
   <si>
@@ -680,6 +677,12 @@
     <t>Смешанный</t>
   </si>
   <si>
+    <t>EUR</t>
+  </si>
+  <si>
+    <t>По результатам оценки через количество потенциальных клиентов базовый доступный объем рынка составляет ориентировочно [SAM] EUR в год, а реалистично достижимый объем для нового бизнеса составляет [SOM] EUR в год. Оценка является сценарной и требует проверки через фактические данные о клиентах, конкурентах, рекламных каналах, Similarweb, поисковом спросе и платежеспособности целевых сегментов.</t>
+  </si>
+  <si>
     <t>TableMind: онлайн-сервис независимой проверки (аудита) Excel-моделей</t>
   </si>
   <si>
@@ -693,9 +696,6 @@
   </si>
   <si>
     <t>B2B и B2C (профессионалы и малый бизнес), подписка freemium</t>
-  </si>
-  <si>
-    <t>EUR</t>
   </si>
   <si>
     <t>Курс НБРБ 03.10.2026: 1 EUR = 3,3860 BYN</t>
@@ -1165,7 +1165,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-694F-40E1-997D-0239D1B8EC5D}"/>
+              <c16:uniqueId val="{00000000-1EF8-4E16-9499-9C457E25BD31}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1231,7 +1231,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-694F-40E1-997D-0239D1B8EC5D}"/>
+              <c16:uniqueId val="{00000001-1EF8-4E16-9499-9C457E25BD31}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1397,7 +1397,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-3ED5-4A04-B558-7E7D27316634}"/>
+              <c16:uniqueId val="{00000000-43EC-4A59-B285-BBB33AFF0673}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1445,7 +1445,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-3ED5-4A04-B558-7E7D27316634}"/>
+              <c16:uniqueId val="{00000001-43EC-4A59-B285-BBB33AFF0673}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1493,7 +1493,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-3ED5-4A04-B558-7E7D27316634}"/>
+              <c16:uniqueId val="{00000002-43EC-4A59-B285-BBB33AFF0673}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7733,7 +7733,7 @@
         <v>53</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>54</v>
@@ -7769,7 +7769,7 @@
         <v>56</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>57</v>
@@ -7805,7 +7805,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>60</v>
@@ -7841,7 +7841,7 @@
         <v>62</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>63</v>
@@ -7877,7 +7877,7 @@
         <v>65</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>66</v>
@@ -7913,7 +7913,7 @@
         <v>68</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>218</v>
@@ -37239,7 +37239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0F1359F6-991C-4F4E-9624-B82D7495C786}</x14:id>
+          <x14:id>{8A6A4B80-A104-49C0-A30B-44ECAA3B4221}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37253,7 +37253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5AF3E2CD-A54F-49F0-955E-AD4F5CD9F574}</x14:id>
+          <x14:id>{67CB3220-67BC-45D2-A768-63B648F902A6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37285,7 +37285,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{82670BB8-7A48-4638-882E-45A10998687B}</x14:id>
+          <x14:id>{F1C43D3F-C8F1-4E58-9306-0FA22557A6EF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37299,7 +37299,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{62E9F17A-C996-41EF-986B-E09180F6B3FD}</x14:id>
+          <x14:id>{7DCF60C4-2602-434A-A4E2-3476257434EA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37331,7 +37331,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F2E11A1B-BB3C-4D87-B1C9-E3771FC5C4BC}</x14:id>
+          <x14:id>{50AFAEA6-C443-4EE5-B08E-E6559F9B2562}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37345,7 +37345,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{19DD2E6F-F9E0-400B-8D83-9A70D5A0D7CF}</x14:id>
+          <x14:id>{6E6EACC2-9170-4E1E-AD32-D05338C057CE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37377,7 +37377,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4CAA12EC-D22E-47C8-8F6D-F8269CB46114}</x14:id>
+          <x14:id>{218155CF-DEB4-4A5C-8934-A03D900670C4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37391,7 +37391,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E5A711C8-750A-4E7B-A932-1EAE65A353FC}</x14:id>
+          <x14:id>{6CD3A58A-8035-4EDA-AC2E-D93D33FAC397}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37423,7 +37423,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F6BB9F28-FB0D-46F9-BBD4-EE0BAB036DDB}</x14:id>
+          <x14:id>{A33DC3DD-3F0F-4631-A146-6B3231AEF94C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37437,7 +37437,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C6F8082E-AEBD-4407-AA61-464BDE36823D}</x14:id>
+          <x14:id>{7F7999C3-33E5-469F-8B3E-0EF9F985D1E2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37469,7 +37469,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5C3FA386-FBFD-43EC-BEC4-C231ABF02710}</x14:id>
+          <x14:id>{9C9B158D-699F-41EC-8FF7-08F84A7B63C7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37483,7 +37483,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{40ED7FC0-2EDA-4B13-BBAF-F84A2DB02224}</x14:id>
+          <x14:id>{C895CC77-9EE2-41FF-945E-5A46FC0D4BFA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37515,7 +37515,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{11505EF9-0401-43AA-822D-3ACE70E665ED}</x14:id>
+          <x14:id>{085AC320-CFBA-41C9-8F51-860055D28591}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37529,7 +37529,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2C856E50-25F3-4C0A-A214-3CEF1D5F734D}</x14:id>
+          <x14:id>{C9DF7F37-551B-4340-8CED-2F29928BBECE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37564,7 +37564,7 @@
           <xm:sqref>O4:O5 O13:O15</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0F1359F6-991C-4F4E-9624-B82D7495C786}">
+          <x14:cfRule type="dataBar" id="{8A6A4B80-A104-49C0-A30B-44ECAA3B4221}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37575,7 +37575,7 @@
           <xm:sqref>I6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5AF3E2CD-A54F-49F0-955E-AD4F5CD9F574}">
+          <x14:cfRule type="dataBar" id="{67CB3220-67BC-45D2-A768-63B648F902A6}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37586,7 +37586,7 @@
           <xm:sqref>O6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{82670BB8-7A48-4638-882E-45A10998687B}">
+          <x14:cfRule type="dataBar" id="{F1C43D3F-C8F1-4E58-9306-0FA22557A6EF}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37597,7 +37597,7 @@
           <xm:sqref>I7</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{62E9F17A-C996-41EF-986B-E09180F6B3FD}">
+          <x14:cfRule type="dataBar" id="{7DCF60C4-2602-434A-A4E2-3476257434EA}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37608,7 +37608,7 @@
           <xm:sqref>O7</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F2E11A1B-BB3C-4D87-B1C9-E3771FC5C4BC}">
+          <x14:cfRule type="dataBar" id="{50AFAEA6-C443-4EE5-B08E-E6559F9B2562}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37619,7 +37619,7 @@
           <xm:sqref>I8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{19DD2E6F-F9E0-400B-8D83-9A70D5A0D7CF}">
+          <x14:cfRule type="dataBar" id="{6E6EACC2-9170-4E1E-AD32-D05338C057CE}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37630,7 +37630,7 @@
           <xm:sqref>O8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4CAA12EC-D22E-47C8-8F6D-F8269CB46114}">
+          <x14:cfRule type="dataBar" id="{218155CF-DEB4-4A5C-8934-A03D900670C4}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37641,7 +37641,7 @@
           <xm:sqref>I9</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E5A711C8-750A-4E7B-A932-1EAE65A353FC}">
+          <x14:cfRule type="dataBar" id="{6CD3A58A-8035-4EDA-AC2E-D93D33FAC397}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37652,7 +37652,7 @@
           <xm:sqref>O9</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F6BB9F28-FB0D-46F9-BBD4-EE0BAB036DDB}">
+          <x14:cfRule type="dataBar" id="{A33DC3DD-3F0F-4631-A146-6B3231AEF94C}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37663,7 +37663,7 @@
           <xm:sqref>I10</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C6F8082E-AEBD-4407-AA61-464BDE36823D}">
+          <x14:cfRule type="dataBar" id="{7F7999C3-33E5-469F-8B3E-0EF9F985D1E2}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37674,7 +37674,7 @@
           <xm:sqref>O10</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5C3FA386-FBFD-43EC-BEC4-C231ABF02710}">
+          <x14:cfRule type="dataBar" id="{9C9B158D-699F-41EC-8FF7-08F84A7B63C7}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37685,7 +37685,7 @@
           <xm:sqref>I11</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{40ED7FC0-2EDA-4B13-BBAF-F84A2DB02224}">
+          <x14:cfRule type="dataBar" id="{C895CC77-9EE2-41FF-945E-5A46FC0D4BFA}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37696,7 +37696,7 @@
           <xm:sqref>O11</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{11505EF9-0401-43AA-822D-3ACE70E665ED}">
+          <x14:cfRule type="dataBar" id="{085AC320-CFBA-41C9-8F51-860055D28591}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37707,7 +37707,7 @@
           <xm:sqref>I12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2C856E50-25F3-4C0A-A214-3CEF1D5F734D}">
+          <x14:cfRule type="dataBar" id="{C9DF7F37-551B-4340-8CED-2F29928BBECE}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -38437,7 +38437,7 @@
     </row>
     <row r="20" spans="1:26">
       <c r="A20" s="18" t="s">
-        <v>189</v>
+        <v>212</v>
       </c>
       <c r="B20" s="18"/>
       <c r="C20" s="18"/>
@@ -43535,7 +43535,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="17.649999999999999">
       <c r="A1" s="16" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -43593,25 +43593,25 @@
     </row>
     <row r="3" spans="1:26" ht="27.75">
       <c r="A3" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>195</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>196</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>51</v>
@@ -43681,7 +43681,7 @@
     </row>
     <row r="5" spans="1:26" ht="40.5">
       <c r="A5" s="10" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>273</v>
@@ -43696,7 +43696,7 @@
         <v>46298</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G5" s="10" t="s">
         <v>108</v>
@@ -43725,7 +43725,7 @@
     </row>
     <row r="6" spans="1:26" ht="27">
       <c r="A6" s="10" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>276</v>
@@ -43740,7 +43740,7 @@
         <v>46298</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G6" s="10" t="s">
         <v>107</v>
@@ -43769,10 +43769,10 @@
     </row>
     <row r="7" spans="1:26" ht="40.5">
       <c r="A7" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>201</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>202</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>279</v>
@@ -43784,7 +43784,7 @@
         <v>46298</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>107</v>
@@ -43857,22 +43857,22 @@
     </row>
     <row r="9" spans="1:26" ht="27">
       <c r="A9" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="B9" s="10" t="s">
         <v>203</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>204</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>285</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E9" s="10">
         <v>46298</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G9" s="10" t="s">
         <v>107</v>
@@ -49289,7 +49289,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="17.649999999999999">
       <c r="A1" s="16" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -49350,10 +49350,10 @@
         <v>92</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>195</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>196</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>112</v>
@@ -49386,10 +49386,10 @@
         <v>106</v>
       </c>
       <c r="B4" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>207</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>208</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>119</v>
@@ -49419,10 +49419,10 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>107</v>
@@ -49455,10 +49455,10 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" s="9" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>108</v>
@@ -49491,7 +49491,7 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>109</v>

</xml_diff>

<commit_message>
audit: fix title page overflow, dashes, source citation, stale statuses, third-person wording, Excel cells, README/plans; rebuild all
</commit_message>
<xml_diff>
--- a/ЛР2-3_Объем_рынка/Excel/ЛР2-3_1_потенциальные_клиенты_TableMind.xlsx
+++ b/ЛР2-3_Объем_рынка/Excel/ЛР2-3_1_потенциальные_клиенты_TableMind.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-continuation-3ab569\ЛР2-3_Объем_рынка\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-continuation-57ce20\ЛР2-3_Объем_рынка\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ED63552-C1B6-4CDF-B6C1-CFE528702DBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F86586CE-0B0C-45B4-BDD4-940AB2D49475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="368" yWindow="368" windowWidth="12022" windowHeight="10972" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2205" yWindow="458" windowWidth="12022" windowHeight="10972" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Методика" sheetId="1" r:id="rId1"/>
@@ -701,9 +701,6 @@
     <t>Курс НБРБ 03.10.2026: 1 EUR = 3,3860 BYN</t>
   </si>
   <si>
-    <t>Р. В. Земляник, гр. 60131</t>
-  </si>
-  <si>
     <t>Финансовые аналитики и FP&amp;A</t>
   </si>
   <si>
@@ -900,6 +897,9 @@
   </si>
   <si>
     <t>Similarweb Pro (пробный доступ), 06-08.2026</t>
+  </si>
+  <si>
+    <t>Р. В. Земляник, гр. 60121</t>
   </si>
 </sst>
 </file>
@@ -8021,7 +8021,7 @@
         <v>76</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>219</v>
+        <v>285</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>77</v>
@@ -13493,13 +13493,13 @@
     </row>
     <row r="4" spans="1:26" ht="27">
       <c r="A4" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="C4" s="10" t="s">
         <v>221</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>222</v>
       </c>
       <c r="D4" s="12">
         <v>1218525</v>
@@ -13545,7 +13545,7 @@
         <v>107</v>
       </c>
       <c r="Q4" s="10" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="R4" s="9"/>
       <c r="S4" s="9"/>
@@ -13559,13 +13559,13 @@
     </row>
     <row r="5" spans="1:26" ht="27">
       <c r="A5" s="10" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B5" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>221</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>222</v>
       </c>
       <c r="D5" s="12">
         <v>4386800</v>
@@ -13611,7 +13611,7 @@
         <v>107</v>
       </c>
       <c r="Q5" s="10" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R5" s="9"/>
       <c r="S5" s="9"/>
@@ -13625,13 +13625,13 @@
     </row>
     <row r="6" spans="1:26" ht="27">
       <c r="A6" s="10" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B6" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>221</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>222</v>
       </c>
       <c r="D6" s="12">
         <v>2962025</v>
@@ -13677,7 +13677,7 @@
         <v>108</v>
       </c>
       <c r="Q6" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="R6" s="9"/>
       <c r="S6" s="9"/>
@@ -13691,13 +13691,13 @@
     </row>
     <row r="7" spans="1:26" ht="27">
       <c r="A7" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>228</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>229</v>
       </c>
       <c r="D7" s="12">
         <v>17415635</v>
@@ -13743,7 +13743,7 @@
         <v>108</v>
       </c>
       <c r="Q7" s="10" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="R7" s="9"/>
       <c r="S7" s="9"/>
@@ -13757,13 +13757,13 @@
     </row>
     <row r="8" spans="1:26">
       <c r="A8" s="10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>106</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D8" s="12">
         <v>0</v>
@@ -13809,7 +13809,7 @@
         <v>109</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="R8" s="9"/>
       <c r="S8" s="9"/>
@@ -13823,13 +13823,13 @@
     </row>
     <row r="9" spans="1:26">
       <c r="A9" s="10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>106</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D9" s="12">
         <v>0</v>
@@ -13875,7 +13875,7 @@
         <v>109</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="R9" s="9"/>
       <c r="S9" s="9"/>
@@ -13889,13 +13889,13 @@
     </row>
     <row r="10" spans="1:26">
       <c r="A10" s="10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>106</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D10" s="12">
         <v>0</v>
@@ -13941,7 +13941,7 @@
         <v>109</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="R10" s="9"/>
       <c r="S10" s="9"/>
@@ -19544,7 +19544,7 @@
         <v>5040.4489902720006</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L4" s="9"/>
       <c r="M4" s="9"/>
@@ -19650,7 +19650,7 @@
         <v>219977.79505794571</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="L6" s="9"/>
       <c r="M6" s="9"/>
@@ -31007,13 +31007,13 @@
     </row>
     <row r="4" spans="1:26" ht="27">
       <c r="A4" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>236</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="C4" s="10" t="s">
         <v>237</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>238</v>
       </c>
       <c r="D4" s="12">
         <v>154111</v>
@@ -31022,7 +31022,7 @@
         <v>0.26539999999999997</v>
       </c>
       <c r="F4" s="12">
-        <f>D4*E4</f>
+        <f t="shared" ref="F4:F15" si="0">D4*E4</f>
         <v>40901.059399999998</v>
       </c>
       <c r="G4" s="13">
@@ -31032,7 +31032,7 @@
         <v>0.85</v>
       </c>
       <c r="I4" s="12">
-        <f>F4*G4*H4</f>
+        <f t="shared" ref="I4:I15" si="1">F4*G4*H4</f>
         <v>12168.065171499999</v>
       </c>
       <c r="J4" s="15">
@@ -31045,15 +31045,15 @@
         <v>100.575</v>
       </c>
       <c r="M4" s="12">
-        <f>I4*J4*K4</f>
+        <f t="shared" ref="M4:M15" si="2">I4*J4*K4</f>
         <v>24.336130342999997</v>
       </c>
       <c r="N4" s="12">
-        <f>M4*L4</f>
+        <f t="shared" ref="N4:N15" si="3">M4*L4</f>
         <v>2447.606309247225</v>
       </c>
       <c r="O4" s="12">
-        <f>N4*12</f>
+        <f t="shared" ref="O4:O15" si="4">N4*12</f>
         <v>29371.2757109667</v>
       </c>
       <c r="P4" s="9"/>
@@ -31070,13 +31070,13 @@
     </row>
     <row r="5" spans="1:26" ht="27">
       <c r="A5" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>239</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="C5" s="10" t="s">
         <v>240</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>241</v>
       </c>
       <c r="D5" s="12">
         <v>35325</v>
@@ -31085,7 +31085,7 @@
         <v>0.4395</v>
       </c>
       <c r="F5" s="12">
-        <f>D5*E5</f>
+        <f t="shared" si="0"/>
         <v>15525.3375</v>
       </c>
       <c r="G5" s="13">
@@ -31095,7 +31095,7 @@
         <v>0.85</v>
       </c>
       <c r="I5" s="12">
-        <f>F5*G5*H5</f>
+        <f t="shared" si="1"/>
         <v>10557.229499999999</v>
       </c>
       <c r="J5" s="15">
@@ -31108,15 +31108,15 @@
         <v>100.575</v>
       </c>
       <c r="M5" s="12">
-        <f>I5*J5*K5</f>
+        <f t="shared" si="2"/>
         <v>21.114459</v>
       </c>
       <c r="N5" s="12">
-        <f>M5*L5</f>
+        <f t="shared" si="3"/>
         <v>2123.5867139249999</v>
       </c>
       <c r="O5" s="12">
-        <f>N5*12</f>
+        <f t="shared" si="4"/>
         <v>25483.040567099997</v>
       </c>
       <c r="P5" s="9"/>
@@ -31133,13 +31133,13 @@
     </row>
     <row r="6" spans="1:26" ht="27">
       <c r="A6" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>242</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="C6" s="10" t="s">
         <v>243</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>244</v>
       </c>
       <c r="D6" s="12">
         <v>241737</v>
@@ -31148,7 +31148,7 @@
         <v>0.1091</v>
       </c>
       <c r="F6" s="12">
-        <f>D6*E6</f>
+        <f t="shared" si="0"/>
         <v>26373.506700000002</v>
       </c>
       <c r="G6" s="13">
@@ -31158,7 +31158,7 @@
         <v>0.85</v>
       </c>
       <c r="I6" s="12">
-        <f>F6*G6*H6</f>
+        <f t="shared" si="1"/>
         <v>3362.6221042500001</v>
       </c>
       <c r="J6" s="15">
@@ -31171,15 +31171,15 @@
         <v>100.575</v>
       </c>
       <c r="M6" s="12">
-        <f>I6*J6*K6</f>
+        <f t="shared" si="2"/>
         <v>6.7252442085000004</v>
       </c>
       <c r="N6" s="12">
-        <f>M6*L6</f>
+        <f t="shared" si="3"/>
         <v>676.39143626988755</v>
       </c>
       <c r="O6" s="12">
-        <f>N6*12</f>
+        <f t="shared" si="4"/>
         <v>8116.697235238651</v>
       </c>
       <c r="P6" s="9"/>
@@ -31196,13 +31196,13 @@
     </row>
     <row r="7" spans="1:26" ht="27">
       <c r="A7" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>245</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="C7" s="10" t="s">
         <v>246</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>247</v>
       </c>
       <c r="D7" s="12">
         <v>202178</v>
@@ -31211,7 +31211,7 @@
         <v>0.16220000000000001</v>
       </c>
       <c r="F7" s="12">
-        <f>D7*E7</f>
+        <f t="shared" si="0"/>
         <v>32793.2716</v>
       </c>
       <c r="G7" s="13">
@@ -31221,7 +31221,7 @@
         <v>0.85</v>
       </c>
       <c r="I7" s="12">
-        <f>F7*G7*H7</f>
+        <f t="shared" si="1"/>
         <v>8362.2842579999997</v>
       </c>
       <c r="J7" s="15">
@@ -31234,15 +31234,15 @@
         <v>100.575</v>
       </c>
       <c r="M7" s="12">
-        <f>I7*J7*K7</f>
+        <f t="shared" si="2"/>
         <v>16.724568516000001</v>
       </c>
       <c r="N7" s="12">
-        <f>M7*L7</f>
+        <f t="shared" si="3"/>
         <v>1682.0734784967001</v>
       </c>
       <c r="O7" s="12">
-        <f>N7*12</f>
+        <f t="shared" si="4"/>
         <v>20184.881741960402</v>
       </c>
       <c r="P7" s="9"/>
@@ -31259,13 +31259,13 @@
     </row>
     <row r="8" spans="1:26" ht="27">
       <c r="A8" s="10" t="s">
+        <v>247</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="C8" s="10" t="s">
         <v>249</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>250</v>
       </c>
       <c r="D8" s="12">
         <v>14688</v>
@@ -31274,7 +31274,7 @@
         <v>0.95979999999999999</v>
       </c>
       <c r="F8" s="12">
-        <f>D8*E8</f>
+        <f t="shared" si="0"/>
         <v>14097.5424</v>
       </c>
       <c r="G8" s="13">
@@ -31284,7 +31284,7 @@
         <v>0.8</v>
       </c>
       <c r="I8" s="12">
-        <f>F8*G8*H8</f>
+        <f t="shared" si="1"/>
         <v>5639.0169600000008</v>
       </c>
       <c r="J8" s="15">
@@ -31297,15 +31297,15 @@
         <v>100.575</v>
       </c>
       <c r="M8" s="12">
-        <f>I8*J8*K8</f>
+        <f t="shared" si="2"/>
         <v>11.278033920000002</v>
       </c>
       <c r="N8" s="12">
-        <f>M8*L8</f>
+        <f t="shared" si="3"/>
         <v>1134.2882615040003</v>
       </c>
       <c r="O8" s="12">
-        <f>N8*12</f>
+        <f t="shared" si="4"/>
         <v>13611.459138048003</v>
       </c>
       <c r="P8" s="9"/>
@@ -31322,13 +31322,13 @@
     </row>
     <row r="9" spans="1:26" ht="27">
       <c r="A9" s="10" t="s">
+        <v>250</v>
+      </c>
+      <c r="B9" s="10" t="s">
         <v>251</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>252</v>
-      </c>
       <c r="C9" s="10" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D9" s="12">
         <v>17824</v>
@@ -31337,7 +31337,7 @@
         <v>0.58709999999999996</v>
       </c>
       <c r="F9" s="12">
-        <f>D9*E9</f>
+        <f t="shared" si="0"/>
         <v>10464.470399999998</v>
       </c>
       <c r="G9" s="13">
@@ -31347,7 +31347,7 @@
         <v>0.8</v>
       </c>
       <c r="I9" s="12">
-        <f>F9*G9*H9</f>
+        <f t="shared" si="1"/>
         <v>6697.2610559999994</v>
       </c>
       <c r="J9" s="15">
@@ -31360,15 +31360,15 @@
         <v>100.575</v>
       </c>
       <c r="M9" s="12">
-        <f>I9*J9*K9</f>
+        <f t="shared" si="2"/>
         <v>13.394522111999999</v>
       </c>
       <c r="N9" s="12">
-        <f>M9*L9</f>
+        <f t="shared" si="3"/>
         <v>1347.1540614143998</v>
       </c>
       <c r="O9" s="12">
-        <f>N9*12</f>
+        <f t="shared" si="4"/>
         <v>16165.848736972799</v>
       </c>
       <c r="P9" s="9"/>
@@ -31385,13 +31385,13 @@
     </row>
     <row r="10" spans="1:26" ht="27">
       <c r="A10" s="10" t="s">
+        <v>252</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>253</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>254</v>
-      </c>
       <c r="C10" s="10" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D10" s="12">
         <v>292214</v>
@@ -31400,7 +31400,7 @@
         <v>9.6499999999999989E-2</v>
       </c>
       <c r="F10" s="12">
-        <f>D10*E10</f>
+        <f t="shared" si="0"/>
         <v>28198.650999999998</v>
       </c>
       <c r="G10" s="13">
@@ -31410,7 +31410,7 @@
         <v>0.8</v>
       </c>
       <c r="I10" s="12">
-        <f>F10*G10*H10</f>
+        <f t="shared" si="1"/>
         <v>6767.6762399999998</v>
       </c>
       <c r="J10" s="15">
@@ -31423,15 +31423,15 @@
         <v>100.575</v>
       </c>
       <c r="M10" s="12">
-        <f>I10*J10*K10</f>
+        <f t="shared" si="2"/>
         <v>13.53535248</v>
       </c>
       <c r="N10" s="12">
-        <f>M10*L10</f>
+        <f t="shared" si="3"/>
         <v>1361.318075676</v>
       </c>
       <c r="O10" s="12">
-        <f>N10*12</f>
+        <f t="shared" si="4"/>
         <v>16335.816908112</v>
       </c>
       <c r="P10" s="9"/>
@@ -31448,13 +31448,13 @@
     </row>
     <row r="11" spans="1:26" ht="27">
       <c r="A11" s="10" t="s">
+        <v>254</v>
+      </c>
+      <c r="B11" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>256</v>
-      </c>
       <c r="C11" s="10" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D11" s="12">
         <v>116617</v>
@@ -31463,7 +31463,7 @@
         <v>0.18229999999999999</v>
       </c>
       <c r="F11" s="12">
-        <f>D11*E11</f>
+        <f t="shared" si="0"/>
         <v>21259.2791</v>
       </c>
       <c r="G11" s="13">
@@ -31473,7 +31473,7 @@
         <v>0.85</v>
       </c>
       <c r="I11" s="12">
-        <f>F11*G11*H11</f>
+        <f t="shared" si="1"/>
         <v>4517.5968087499996</v>
       </c>
       <c r="J11" s="15">
@@ -31486,15 +31486,15 @@
         <v>100.575</v>
       </c>
       <c r="M11" s="12">
-        <f>I11*J11*K11</f>
+        <f t="shared" si="2"/>
         <v>9.0351936174999992</v>
       </c>
       <c r="N11" s="12">
-        <f>M11*L11</f>
+        <f t="shared" si="3"/>
         <v>908.71459808006239</v>
       </c>
       <c r="O11" s="12">
-        <f>N11*12</f>
+        <f t="shared" si="4"/>
         <v>10904.575176960749</v>
       </c>
       <c r="P11" s="9"/>
@@ -31511,13 +31511,13 @@
     </row>
     <row r="12" spans="1:26" ht="27">
       <c r="A12" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="C12" s="10" t="s">
         <v>258</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>259</v>
       </c>
       <c r="D12" s="12">
         <v>222359</v>
@@ -31526,7 +31526,7 @@
         <v>0.76359999999999995</v>
       </c>
       <c r="F12" s="12">
-        <f>D12*E12</f>
+        <f t="shared" si="0"/>
         <v>169793.33239999998</v>
       </c>
       <c r="G12" s="13">
@@ -31536,7 +31536,7 @@
         <v>0.9</v>
       </c>
       <c r="I12" s="12">
-        <f>F12*G12*H12</f>
+        <f t="shared" si="1"/>
         <v>22922.099873999996</v>
       </c>
       <c r="J12" s="15">
@@ -31549,15 +31549,15 @@
         <v>100.575</v>
       </c>
       <c r="M12" s="12">
-        <f>I12*J12*K12</f>
+        <f t="shared" si="2"/>
         <v>45.844199747999994</v>
       </c>
       <c r="N12" s="12">
-        <f>M12*L12</f>
+        <f t="shared" si="3"/>
         <v>4610.7803896550995</v>
       </c>
       <c r="O12" s="12">
-        <f>N12*12</f>
+        <f t="shared" si="4"/>
         <v>55329.364675861194</v>
       </c>
       <c r="P12" s="9"/>
@@ -31574,13 +31574,13 @@
     </row>
     <row r="13" spans="1:26" ht="27">
       <c r="A13" s="10" t="s">
+        <v>259</v>
+      </c>
+      <c r="B13" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="C13" s="10" t="s">
         <v>261</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>262</v>
       </c>
       <c r="D13" s="12">
         <v>701540</v>
@@ -31589,7 +31589,7 @@
         <v>8.199999999999999E-2</v>
       </c>
       <c r="F13" s="12">
-        <f>D13*E13</f>
+        <f t="shared" si="0"/>
         <v>57526.279999999992</v>
       </c>
       <c r="G13" s="13">
@@ -31599,7 +31599,7 @@
         <v>0.85</v>
       </c>
       <c r="I13" s="12">
-        <f>F13*G13*H13</f>
+        <f t="shared" si="1"/>
         <v>4889.7338</v>
       </c>
       <c r="J13" s="15">
@@ -31612,15 +31612,15 @@
         <v>100.575</v>
       </c>
       <c r="M13" s="12">
-        <f>I13*J13*K13</f>
+        <f t="shared" si="2"/>
         <v>9.7794676000000003</v>
       </c>
       <c r="N13" s="12">
-        <f>M13*L13</f>
+        <f t="shared" si="3"/>
         <v>983.56995387000006</v>
       </c>
       <c r="O13" s="12">
-        <f>N13*12</f>
+        <f t="shared" si="4"/>
         <v>11802.839446440001</v>
       </c>
       <c r="P13" s="9"/>
@@ -31637,13 +31637,13 @@
     </row>
     <row r="14" spans="1:26" ht="27">
       <c r="A14" s="10" t="s">
+        <v>262</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>263</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>264</v>
-      </c>
       <c r="C14" s="10" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D14" s="12">
         <v>1935</v>
@@ -31652,7 +31652,7 @@
         <v>0.89460000000000006</v>
       </c>
       <c r="F14" s="12">
-        <f>D14*E14</f>
+        <f t="shared" si="0"/>
         <v>1731.0510000000002</v>
       </c>
       <c r="G14" s="13">
@@ -31662,7 +31662,7 @@
         <v>0.6</v>
       </c>
       <c r="I14" s="12">
-        <f>F14*G14*H14</f>
+        <f t="shared" si="1"/>
         <v>830.90448000000004</v>
       </c>
       <c r="J14" s="15">
@@ -31675,15 +31675,15 @@
         <v>100.575</v>
       </c>
       <c r="M14" s="12">
-        <f>I14*J14*K14</f>
+        <f t="shared" si="2"/>
         <v>1.6618089600000001</v>
       </c>
       <c r="N14" s="12">
-        <f>M14*L14</f>
+        <f t="shared" si="3"/>
         <v>167.13643615200002</v>
       </c>
       <c r="O14" s="12">
-        <f>N14*12</f>
+        <f t="shared" si="4"/>
         <v>2005.6372338240003</v>
       </c>
       <c r="P14" s="9"/>
@@ -31700,13 +31700,13 @@
     </row>
     <row r="15" spans="1:26" ht="27">
       <c r="A15" s="10" t="s">
+        <v>264</v>
+      </c>
+      <c r="B15" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="C15" s="10" t="s">
         <v>266</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>267</v>
       </c>
       <c r="D15" s="12">
         <v>5522</v>
@@ -31715,7 +31715,7 @@
         <v>0.47520000000000001</v>
       </c>
       <c r="F15" s="12">
-        <f>D15*E15</f>
+        <f t="shared" si="0"/>
         <v>2624.0544</v>
       </c>
       <c r="G15" s="13">
@@ -31725,7 +31725,7 @@
         <v>0.6</v>
       </c>
       <c r="I15" s="12">
-        <f>F15*G15*H15</f>
+        <f t="shared" si="1"/>
         <v>472.329792</v>
       </c>
       <c r="J15" s="15">
@@ -31738,15 +31738,15 @@
         <v>100.575</v>
       </c>
       <c r="M15" s="12">
-        <f>I15*J15*K15</f>
+        <f t="shared" si="2"/>
         <v>0.94465958400000005</v>
       </c>
       <c r="N15" s="12">
-        <f>M15*L15</f>
+        <f t="shared" si="3"/>
         <v>95.009137660800008</v>
       </c>
       <c r="O15" s="12">
-        <f>N15*12</f>
+        <f t="shared" si="4"/>
         <v>1140.1096519296002</v>
       </c>
       <c r="P15" s="9"/>
@@ -38049,7 +38049,7 @@
       <c r="Y8" s="9"/>
       <c r="Z8" s="9"/>
     </row>
-    <row r="9" spans="1:26" ht="27">
+    <row r="9" spans="1:26">
       <c r="A9" s="10" t="s">
         <v>139</v>
       </c>
@@ -43640,25 +43640,25 @@
         <v>80</v>
       </c>
       <c r="B4" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>268</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="D4" s="10" t="s">
         <v>269</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>270</v>
       </c>
       <c r="E4" s="10">
         <v>46298</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="G4" s="10" t="s">
         <v>107</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
@@ -43684,13 +43684,13 @@
         <v>197</v>
       </c>
       <c r="B5" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="D5" s="10" t="s">
         <v>274</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>275</v>
       </c>
       <c r="E5" s="10">
         <v>46298</v>
@@ -43702,7 +43702,7 @@
         <v>108</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I5" s="9"/>
       <c r="J5" s="9"/>
@@ -43728,13 +43728,13 @@
         <v>199</v>
       </c>
       <c r="B6" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>276</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="D6" s="10" t="s">
         <v>277</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>278</v>
       </c>
       <c r="E6" s="10">
         <v>46298</v>
@@ -43746,7 +43746,7 @@
         <v>107</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I6" s="9"/>
       <c r="J6" s="9"/>
@@ -43775,10 +43775,10 @@
         <v>201</v>
       </c>
       <c r="C7" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>279</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>280</v>
       </c>
       <c r="E7" s="10">
         <v>46298</v>
@@ -43790,7 +43790,7 @@
         <v>107</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
@@ -43816,25 +43816,25 @@
         <v>84</v>
       </c>
       <c r="B8" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="D8" s="10" t="s">
         <v>282</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>283</v>
       </c>
       <c r="E8" s="10">
         <v>46298</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>107</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I8" s="9"/>
       <c r="J8" s="9"/>
@@ -43863,7 +43863,7 @@
         <v>203</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>204</v>
@@ -43878,7 +43878,7 @@
         <v>107</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="9"/>

</xml_diff>

<commit_message>
audit: fix inaccuracies against lab conditions, regenerate figures, reports and PDFs (final 255 pages)
</commit_message>
<xml_diff>
--- a/ЛР2-3_Объем_рынка/Excel/ЛР2-3_1_потенциальные_клиенты_TableMind.xlsx
+++ b/ЛР2-3_Объем_рынка/Excel/ЛР2-3_1_потенциальные_клиенты_TableMind.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-continuation-57ce20\ЛР2-3_Объем_рынка\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-project-continuation-447426\ЛР2-3_Объем_рынка\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F86586CE-0B0C-45B4-BDD4-940AB2D49475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F6D6D31-175C-458B-B2AC-50134AF29623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="458" windowWidth="12022" windowHeight="10972" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
     <sheet name="07_Источники" sheetId="8" r:id="rId8"/>
     <sheet name="08_Справочник" sheetId="9" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="191029" refMode="R1C1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -701,6 +701,9 @@
     <t>Курс НБРБ 03.10.2026: 1 EUR = 3,3860 BYN</t>
   </si>
   <si>
+    <t>Р. В. Земляник, гр. 60131</t>
+  </si>
+  <si>
     <t>Финансовые аналитики и FP&amp;A</t>
   </si>
   <si>
@@ -897,9 +900,6 @@
   </si>
   <si>
     <t>Similarweb Pro (пробный доступ), 06-08.2026</t>
-  </si>
-  <si>
-    <t>Р. В. Земляник, гр. 60121</t>
   </si>
 </sst>
 </file>
@@ -1165,7 +1165,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-1EF8-4E16-9499-9C457E25BD31}"/>
+              <c16:uniqueId val="{00000000-9F8E-44C6-9199-F3F73541D651}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1231,7 +1231,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-1EF8-4E16-9499-9C457E25BD31}"/>
+              <c16:uniqueId val="{00000001-9F8E-44C6-9199-F3F73541D651}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1397,7 +1397,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-43EC-4A59-B285-BBB33AFF0673}"/>
+              <c16:uniqueId val="{00000000-93DF-4CA0-BFCA-F21826099D95}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1445,7 +1445,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-43EC-4A59-B285-BBB33AFF0673}"/>
+              <c16:uniqueId val="{00000001-93DF-4CA0-BFCA-F21826099D95}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1493,7 +1493,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-43EC-4A59-B285-BBB33AFF0673}"/>
+              <c16:uniqueId val="{00000002-93DF-4CA0-BFCA-F21826099D95}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -8021,7 +8021,7 @@
         <v>76</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>285</v>
+        <v>219</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>77</v>
@@ -13493,13 +13493,13 @@
     </row>
     <row r="4" spans="1:26" ht="27">
       <c r="A4" s="10" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D4" s="12">
         <v>1218525</v>
@@ -13545,7 +13545,7 @@
         <v>107</v>
       </c>
       <c r="Q4" s="10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="R4" s="9"/>
       <c r="S4" s="9"/>
@@ -13559,13 +13559,13 @@
     </row>
     <row r="5" spans="1:26" ht="27">
       <c r="A5" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D5" s="12">
         <v>4386800</v>
@@ -13611,7 +13611,7 @@
         <v>107</v>
       </c>
       <c r="Q5" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="R5" s="9"/>
       <c r="S5" s="9"/>
@@ -13625,13 +13625,13 @@
     </row>
     <row r="6" spans="1:26" ht="27">
       <c r="A6" s="10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D6" s="12">
         <v>2962025</v>
@@ -13677,7 +13677,7 @@
         <v>108</v>
       </c>
       <c r="Q6" s="10" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="R6" s="9"/>
       <c r="S6" s="9"/>
@@ -13691,13 +13691,13 @@
     </row>
     <row r="7" spans="1:26" ht="27">
       <c r="A7" s="10" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D7" s="12">
         <v>17415635</v>
@@ -13743,7 +13743,7 @@
         <v>108</v>
       </c>
       <c r="Q7" s="10" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="R7" s="9"/>
       <c r="S7" s="9"/>
@@ -13757,13 +13757,13 @@
     </row>
     <row r="8" spans="1:26">
       <c r="A8" s="10" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>106</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D8" s="12">
         <v>0</v>
@@ -13809,7 +13809,7 @@
         <v>109</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="R8" s="9"/>
       <c r="S8" s="9"/>
@@ -13823,13 +13823,13 @@
     </row>
     <row r="9" spans="1:26">
       <c r="A9" s="10" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>106</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D9" s="12">
         <v>0</v>
@@ -13875,7 +13875,7 @@
         <v>109</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="R9" s="9"/>
       <c r="S9" s="9"/>
@@ -13889,13 +13889,13 @@
     </row>
     <row r="10" spans="1:26">
       <c r="A10" s="10" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>106</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D10" s="12">
         <v>0</v>
@@ -13941,7 +13941,7 @@
         <v>109</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="R10" s="9"/>
       <c r="S10" s="9"/>
@@ -19544,7 +19544,7 @@
         <v>5040.4489902720006</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="L4" s="9"/>
       <c r="M4" s="9"/>
@@ -19650,7 +19650,7 @@
         <v>219977.79505794571</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="L6" s="9"/>
       <c r="M6" s="9"/>
@@ -31007,13 +31007,13 @@
     </row>
     <row r="4" spans="1:26" ht="27">
       <c r="A4" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D4" s="12">
         <v>154111</v>
@@ -31022,7 +31022,7 @@
         <v>0.26539999999999997</v>
       </c>
       <c r="F4" s="12">
-        <f t="shared" ref="F4:F15" si="0">D4*E4</f>
+        <f>D4*E4</f>
         <v>40901.059399999998</v>
       </c>
       <c r="G4" s="13">
@@ -31032,7 +31032,7 @@
         <v>0.85</v>
       </c>
       <c r="I4" s="12">
-        <f t="shared" ref="I4:I15" si="1">F4*G4*H4</f>
+        <f>F4*G4*H4</f>
         <v>12168.065171499999</v>
       </c>
       <c r="J4" s="15">
@@ -31045,15 +31045,15 @@
         <v>100.575</v>
       </c>
       <c r="M4" s="12">
-        <f t="shared" ref="M4:M15" si="2">I4*J4*K4</f>
+        <f>I4*J4*K4</f>
         <v>24.336130342999997</v>
       </c>
       <c r="N4" s="12">
-        <f t="shared" ref="N4:N15" si="3">M4*L4</f>
+        <f>M4*L4</f>
         <v>2447.606309247225</v>
       </c>
       <c r="O4" s="12">
-        <f t="shared" ref="O4:O15" si="4">N4*12</f>
+        <f>N4*12</f>
         <v>29371.2757109667</v>
       </c>
       <c r="P4" s="9"/>
@@ -31070,13 +31070,13 @@
     </row>
     <row r="5" spans="1:26" ht="27">
       <c r="A5" s="10" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D5" s="12">
         <v>35325</v>
@@ -31085,7 +31085,7 @@
         <v>0.4395</v>
       </c>
       <c r="F5" s="12">
-        <f t="shared" si="0"/>
+        <f>D5*E5</f>
         <v>15525.3375</v>
       </c>
       <c r="G5" s="13">
@@ -31095,7 +31095,7 @@
         <v>0.85</v>
       </c>
       <c r="I5" s="12">
-        <f t="shared" si="1"/>
+        <f>F5*G5*H5</f>
         <v>10557.229499999999</v>
       </c>
       <c r="J5" s="15">
@@ -31108,15 +31108,15 @@
         <v>100.575</v>
       </c>
       <c r="M5" s="12">
-        <f t="shared" si="2"/>
+        <f>I5*J5*K5</f>
         <v>21.114459</v>
       </c>
       <c r="N5" s="12">
-        <f t="shared" si="3"/>
+        <f>M5*L5</f>
         <v>2123.5867139249999</v>
       </c>
       <c r="O5" s="12">
-        <f t="shared" si="4"/>
+        <f>N5*12</f>
         <v>25483.040567099997</v>
       </c>
       <c r="P5" s="9"/>
@@ -31133,13 +31133,13 @@
     </row>
     <row r="6" spans="1:26" ht="27">
       <c r="A6" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D6" s="12">
         <v>241737</v>
@@ -31148,7 +31148,7 @@
         <v>0.1091</v>
       </c>
       <c r="F6" s="12">
-        <f t="shared" si="0"/>
+        <f>D6*E6</f>
         <v>26373.506700000002</v>
       </c>
       <c r="G6" s="13">
@@ -31158,7 +31158,7 @@
         <v>0.85</v>
       </c>
       <c r="I6" s="12">
-        <f t="shared" si="1"/>
+        <f>F6*G6*H6</f>
         <v>3362.6221042500001</v>
       </c>
       <c r="J6" s="15">
@@ -31171,15 +31171,15 @@
         <v>100.575</v>
       </c>
       <c r="M6" s="12">
-        <f t="shared" si="2"/>
+        <f>I6*J6*K6</f>
         <v>6.7252442085000004</v>
       </c>
       <c r="N6" s="12">
-        <f t="shared" si="3"/>
+        <f>M6*L6</f>
         <v>676.39143626988755</v>
       </c>
       <c r="O6" s="12">
-        <f t="shared" si="4"/>
+        <f>N6*12</f>
         <v>8116.697235238651</v>
       </c>
       <c r="P6" s="9"/>
@@ -31196,13 +31196,13 @@
     </row>
     <row r="7" spans="1:26" ht="27">
       <c r="A7" s="10" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D7" s="12">
         <v>202178</v>
@@ -31211,7 +31211,7 @@
         <v>0.16220000000000001</v>
       </c>
       <c r="F7" s="12">
-        <f t="shared" si="0"/>
+        <f>D7*E7</f>
         <v>32793.2716</v>
       </c>
       <c r="G7" s="13">
@@ -31221,7 +31221,7 @@
         <v>0.85</v>
       </c>
       <c r="I7" s="12">
-        <f t="shared" si="1"/>
+        <f>F7*G7*H7</f>
         <v>8362.2842579999997</v>
       </c>
       <c r="J7" s="15">
@@ -31234,15 +31234,15 @@
         <v>100.575</v>
       </c>
       <c r="M7" s="12">
-        <f t="shared" si="2"/>
+        <f>I7*J7*K7</f>
         <v>16.724568516000001</v>
       </c>
       <c r="N7" s="12">
-        <f t="shared" si="3"/>
+        <f>M7*L7</f>
         <v>1682.0734784967001</v>
       </c>
       <c r="O7" s="12">
-        <f t="shared" si="4"/>
+        <f>N7*12</f>
         <v>20184.881741960402</v>
       </c>
       <c r="P7" s="9"/>
@@ -31259,13 +31259,13 @@
     </row>
     <row r="8" spans="1:26" ht="27">
       <c r="A8" s="10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D8" s="12">
         <v>14688</v>
@@ -31274,7 +31274,7 @@
         <v>0.95979999999999999</v>
       </c>
       <c r="F8" s="12">
-        <f t="shared" si="0"/>
+        <f>D8*E8</f>
         <v>14097.5424</v>
       </c>
       <c r="G8" s="13">
@@ -31284,7 +31284,7 @@
         <v>0.8</v>
       </c>
       <c r="I8" s="12">
-        <f t="shared" si="1"/>
+        <f>F8*G8*H8</f>
         <v>5639.0169600000008</v>
       </c>
       <c r="J8" s="15">
@@ -31297,15 +31297,15 @@
         <v>100.575</v>
       </c>
       <c r="M8" s="12">
-        <f t="shared" si="2"/>
+        <f>I8*J8*K8</f>
         <v>11.278033920000002</v>
       </c>
       <c r="N8" s="12">
-        <f t="shared" si="3"/>
+        <f>M8*L8</f>
         <v>1134.2882615040003</v>
       </c>
       <c r="O8" s="12">
-        <f t="shared" si="4"/>
+        <f>N8*12</f>
         <v>13611.459138048003</v>
       </c>
       <c r="P8" s="9"/>
@@ -31322,13 +31322,13 @@
     </row>
     <row r="9" spans="1:26" ht="27">
       <c r="A9" s="10" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D9" s="12">
         <v>17824</v>
@@ -31337,7 +31337,7 @@
         <v>0.58709999999999996</v>
       </c>
       <c r="F9" s="12">
-        <f t="shared" si="0"/>
+        <f>D9*E9</f>
         <v>10464.470399999998</v>
       </c>
       <c r="G9" s="13">
@@ -31347,7 +31347,7 @@
         <v>0.8</v>
       </c>
       <c r="I9" s="12">
-        <f t="shared" si="1"/>
+        <f>F9*G9*H9</f>
         <v>6697.2610559999994</v>
       </c>
       <c r="J9" s="15">
@@ -31360,15 +31360,15 @@
         <v>100.575</v>
       </c>
       <c r="M9" s="12">
-        <f t="shared" si="2"/>
+        <f>I9*J9*K9</f>
         <v>13.394522111999999</v>
       </c>
       <c r="N9" s="12">
-        <f t="shared" si="3"/>
+        <f>M9*L9</f>
         <v>1347.1540614143998</v>
       </c>
       <c r="O9" s="12">
-        <f t="shared" si="4"/>
+        <f>N9*12</f>
         <v>16165.848736972799</v>
       </c>
       <c r="P9" s="9"/>
@@ -31385,13 +31385,13 @@
     </row>
     <row r="10" spans="1:26" ht="27">
       <c r="A10" s="10" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D10" s="12">
         <v>292214</v>
@@ -31400,7 +31400,7 @@
         <v>9.6499999999999989E-2</v>
       </c>
       <c r="F10" s="12">
-        <f t="shared" si="0"/>
+        <f>D10*E10</f>
         <v>28198.650999999998</v>
       </c>
       <c r="G10" s="13">
@@ -31410,7 +31410,7 @@
         <v>0.8</v>
       </c>
       <c r="I10" s="12">
-        <f t="shared" si="1"/>
+        <f>F10*G10*H10</f>
         <v>6767.6762399999998</v>
       </c>
       <c r="J10" s="15">
@@ -31423,15 +31423,15 @@
         <v>100.575</v>
       </c>
       <c r="M10" s="12">
-        <f t="shared" si="2"/>
+        <f>I10*J10*K10</f>
         <v>13.53535248</v>
       </c>
       <c r="N10" s="12">
-        <f t="shared" si="3"/>
+        <f>M10*L10</f>
         <v>1361.318075676</v>
       </c>
       <c r="O10" s="12">
-        <f t="shared" si="4"/>
+        <f>N10*12</f>
         <v>16335.816908112</v>
       </c>
       <c r="P10" s="9"/>
@@ -31448,13 +31448,13 @@
     </row>
     <row r="11" spans="1:26" ht="27">
       <c r="A11" s="10" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D11" s="12">
         <v>116617</v>
@@ -31463,7 +31463,7 @@
         <v>0.18229999999999999</v>
       </c>
       <c r="F11" s="12">
-        <f t="shared" si="0"/>
+        <f>D11*E11</f>
         <v>21259.2791</v>
       </c>
       <c r="G11" s="13">
@@ -31473,7 +31473,7 @@
         <v>0.85</v>
       </c>
       <c r="I11" s="12">
-        <f t="shared" si="1"/>
+        <f>F11*G11*H11</f>
         <v>4517.5968087499996</v>
       </c>
       <c r="J11" s="15">
@@ -31486,15 +31486,15 @@
         <v>100.575</v>
       </c>
       <c r="M11" s="12">
-        <f t="shared" si="2"/>
+        <f>I11*J11*K11</f>
         <v>9.0351936174999992</v>
       </c>
       <c r="N11" s="12">
-        <f t="shared" si="3"/>
+        <f>M11*L11</f>
         <v>908.71459808006239</v>
       </c>
       <c r="O11" s="12">
-        <f t="shared" si="4"/>
+        <f>N11*12</f>
         <v>10904.575176960749</v>
       </c>
       <c r="P11" s="9"/>
@@ -31511,13 +31511,13 @@
     </row>
     <row r="12" spans="1:26" ht="27">
       <c r="A12" s="10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D12" s="12">
         <v>222359</v>
@@ -31526,7 +31526,7 @@
         <v>0.76359999999999995</v>
       </c>
       <c r="F12" s="12">
-        <f t="shared" si="0"/>
+        <f>D12*E12</f>
         <v>169793.33239999998</v>
       </c>
       <c r="G12" s="13">
@@ -31536,7 +31536,7 @@
         <v>0.9</v>
       </c>
       <c r="I12" s="12">
-        <f t="shared" si="1"/>
+        <f>F12*G12*H12</f>
         <v>22922.099873999996</v>
       </c>
       <c r="J12" s="15">
@@ -31549,15 +31549,15 @@
         <v>100.575</v>
       </c>
       <c r="M12" s="12">
-        <f t="shared" si="2"/>
+        <f>I12*J12*K12</f>
         <v>45.844199747999994</v>
       </c>
       <c r="N12" s="12">
-        <f t="shared" si="3"/>
+        <f>M12*L12</f>
         <v>4610.7803896550995</v>
       </c>
       <c r="O12" s="12">
-        <f t="shared" si="4"/>
+        <f>N12*12</f>
         <v>55329.364675861194</v>
       </c>
       <c r="P12" s="9"/>
@@ -31574,13 +31574,13 @@
     </row>
     <row r="13" spans="1:26" ht="27">
       <c r="A13" s="10" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D13" s="12">
         <v>701540</v>
@@ -31589,7 +31589,7 @@
         <v>8.199999999999999E-2</v>
       </c>
       <c r="F13" s="12">
-        <f t="shared" si="0"/>
+        <f>D13*E13</f>
         <v>57526.279999999992</v>
       </c>
       <c r="G13" s="13">
@@ -31599,7 +31599,7 @@
         <v>0.85</v>
       </c>
       <c r="I13" s="12">
-        <f t="shared" si="1"/>
+        <f>F13*G13*H13</f>
         <v>4889.7338</v>
       </c>
       <c r="J13" s="15">
@@ -31612,15 +31612,15 @@
         <v>100.575</v>
       </c>
       <c r="M13" s="12">
-        <f t="shared" si="2"/>
+        <f>I13*J13*K13</f>
         <v>9.7794676000000003</v>
       </c>
       <c r="N13" s="12">
-        <f t="shared" si="3"/>
+        <f>M13*L13</f>
         <v>983.56995387000006</v>
       </c>
       <c r="O13" s="12">
-        <f t="shared" si="4"/>
+        <f>N13*12</f>
         <v>11802.839446440001</v>
       </c>
       <c r="P13" s="9"/>
@@ -31637,13 +31637,13 @@
     </row>
     <row r="14" spans="1:26" ht="27">
       <c r="A14" s="10" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D14" s="12">
         <v>1935</v>
@@ -31652,7 +31652,7 @@
         <v>0.89460000000000006</v>
       </c>
       <c r="F14" s="12">
-        <f t="shared" si="0"/>
+        <f>D14*E14</f>
         <v>1731.0510000000002</v>
       </c>
       <c r="G14" s="13">
@@ -31662,7 +31662,7 @@
         <v>0.6</v>
       </c>
       <c r="I14" s="12">
-        <f t="shared" si="1"/>
+        <f>F14*G14*H14</f>
         <v>830.90448000000004</v>
       </c>
       <c r="J14" s="15">
@@ -31675,15 +31675,15 @@
         <v>100.575</v>
       </c>
       <c r="M14" s="12">
-        <f t="shared" si="2"/>
+        <f>I14*J14*K14</f>
         <v>1.6618089600000001</v>
       </c>
       <c r="N14" s="12">
-        <f t="shared" si="3"/>
+        <f>M14*L14</f>
         <v>167.13643615200002</v>
       </c>
       <c r="O14" s="12">
-        <f t="shared" si="4"/>
+        <f>N14*12</f>
         <v>2005.6372338240003</v>
       </c>
       <c r="P14" s="9"/>
@@ -31700,13 +31700,13 @@
     </row>
     <row r="15" spans="1:26" ht="27">
       <c r="A15" s="10" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D15" s="12">
         <v>5522</v>
@@ -31715,7 +31715,7 @@
         <v>0.47520000000000001</v>
       </c>
       <c r="F15" s="12">
-        <f t="shared" si="0"/>
+        <f>D15*E15</f>
         <v>2624.0544</v>
       </c>
       <c r="G15" s="13">
@@ -31725,7 +31725,7 @@
         <v>0.6</v>
       </c>
       <c r="I15" s="12">
-        <f t="shared" si="1"/>
+        <f>F15*G15*H15</f>
         <v>472.329792</v>
       </c>
       <c r="J15" s="15">
@@ -31738,15 +31738,15 @@
         <v>100.575</v>
       </c>
       <c r="M15" s="12">
-        <f t="shared" si="2"/>
+        <f>I15*J15*K15</f>
         <v>0.94465958400000005</v>
       </c>
       <c r="N15" s="12">
-        <f t="shared" si="3"/>
+        <f>M15*L15</f>
         <v>95.009137660800008</v>
       </c>
       <c r="O15" s="12">
-        <f t="shared" si="4"/>
+        <f>N15*12</f>
         <v>1140.1096519296002</v>
       </c>
       <c r="P15" s="9"/>
@@ -37239,7 +37239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8A6A4B80-A104-49C0-A30B-44ECAA3B4221}</x14:id>
+          <x14:id>{19B092F5-97FB-4C0A-9C8C-40ABA9F679B2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37253,7 +37253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{67CB3220-67BC-45D2-A768-63B648F902A6}</x14:id>
+          <x14:id>{BFED631D-F43A-4AB9-9CDC-C75D392666A3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37285,7 +37285,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F1C43D3F-C8F1-4E58-9306-0FA22557A6EF}</x14:id>
+          <x14:id>{8CEF1969-B919-4D8A-B897-7D6D5A37F215}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37299,7 +37299,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7DCF60C4-2602-434A-A4E2-3476257434EA}</x14:id>
+          <x14:id>{D7FF9E30-C39E-4C16-8821-6E9ADD4F048C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37331,7 +37331,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{50AFAEA6-C443-4EE5-B08E-E6559F9B2562}</x14:id>
+          <x14:id>{22A79C03-5308-48FD-92DE-AC368385D5F0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37345,7 +37345,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6E6EACC2-9170-4E1E-AD32-D05338C057CE}</x14:id>
+          <x14:id>{78704DF2-01A5-4F19-9A2D-29E3748B20B2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37377,7 +37377,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{218155CF-DEB4-4A5C-8934-A03D900670C4}</x14:id>
+          <x14:id>{25D83344-C72D-4CA8-B7C2-C73E123B3E99}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37391,7 +37391,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6CD3A58A-8035-4EDA-AC2E-D93D33FAC397}</x14:id>
+          <x14:id>{868DCA10-951C-4065-961D-385D8E9AA796}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37423,7 +37423,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A33DC3DD-3F0F-4631-A146-6B3231AEF94C}</x14:id>
+          <x14:id>{2CFC8904-BE06-4688-966A-50364C9C2093}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37437,7 +37437,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7F7999C3-33E5-469F-8B3E-0EF9F985D1E2}</x14:id>
+          <x14:id>{49EC93E7-804B-4E62-B374-28079E653682}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37469,7 +37469,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9C9B158D-699F-41EC-8FF7-08F84A7B63C7}</x14:id>
+          <x14:id>{2ACA975A-79A2-477D-9FD8-A120D68F07C7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37483,7 +37483,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C895CC77-9EE2-41FF-945E-5A46FC0D4BFA}</x14:id>
+          <x14:id>{37699D38-4C97-4A44-8067-5EE2EC15DEC1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37515,7 +37515,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{085AC320-CFBA-41C9-8F51-860055D28591}</x14:id>
+          <x14:id>{E1717276-8550-4700-8014-924D0A8786E3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37529,7 +37529,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C9DF7F37-551B-4340-8CED-2F29928BBECE}</x14:id>
+          <x14:id>{E14950CF-8344-4F4B-983B-C53705049FF6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37564,7 +37564,7 @@
           <xm:sqref>O4:O5 O13:O15</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8A6A4B80-A104-49C0-A30B-44ECAA3B4221}">
+          <x14:cfRule type="dataBar" id="{19B092F5-97FB-4C0A-9C8C-40ABA9F679B2}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37575,7 +37575,7 @@
           <xm:sqref>I6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{67CB3220-67BC-45D2-A768-63B648F902A6}">
+          <x14:cfRule type="dataBar" id="{BFED631D-F43A-4AB9-9CDC-C75D392666A3}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37586,7 +37586,7 @@
           <xm:sqref>O6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F1C43D3F-C8F1-4E58-9306-0FA22557A6EF}">
+          <x14:cfRule type="dataBar" id="{8CEF1969-B919-4D8A-B897-7D6D5A37F215}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37597,7 +37597,7 @@
           <xm:sqref>I7</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7DCF60C4-2602-434A-A4E2-3476257434EA}">
+          <x14:cfRule type="dataBar" id="{D7FF9E30-C39E-4C16-8821-6E9ADD4F048C}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37608,7 +37608,7 @@
           <xm:sqref>O7</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{50AFAEA6-C443-4EE5-B08E-E6559F9B2562}">
+          <x14:cfRule type="dataBar" id="{22A79C03-5308-48FD-92DE-AC368385D5F0}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37619,7 +37619,7 @@
           <xm:sqref>I8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6E6EACC2-9170-4E1E-AD32-D05338C057CE}">
+          <x14:cfRule type="dataBar" id="{78704DF2-01A5-4F19-9A2D-29E3748B20B2}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37630,7 +37630,7 @@
           <xm:sqref>O8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{218155CF-DEB4-4A5C-8934-A03D900670C4}">
+          <x14:cfRule type="dataBar" id="{25D83344-C72D-4CA8-B7C2-C73E123B3E99}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37641,7 +37641,7 @@
           <xm:sqref>I9</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6CD3A58A-8035-4EDA-AC2E-D93D33FAC397}">
+          <x14:cfRule type="dataBar" id="{868DCA10-951C-4065-961D-385D8E9AA796}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37652,7 +37652,7 @@
           <xm:sqref>O9</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A33DC3DD-3F0F-4631-A146-6B3231AEF94C}">
+          <x14:cfRule type="dataBar" id="{2CFC8904-BE06-4688-966A-50364C9C2093}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37663,7 +37663,7 @@
           <xm:sqref>I10</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7F7999C3-33E5-469F-8B3E-0EF9F985D1E2}">
+          <x14:cfRule type="dataBar" id="{49EC93E7-804B-4E62-B374-28079E653682}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37674,7 +37674,7 @@
           <xm:sqref>O10</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9C9B158D-699F-41EC-8FF7-08F84A7B63C7}">
+          <x14:cfRule type="dataBar" id="{2ACA975A-79A2-477D-9FD8-A120D68F07C7}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37685,7 +37685,7 @@
           <xm:sqref>I11</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C895CC77-9EE2-41FF-945E-5A46FC0D4BFA}">
+          <x14:cfRule type="dataBar" id="{37699D38-4C97-4A44-8067-5EE2EC15DEC1}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37696,7 +37696,7 @@
           <xm:sqref>O11</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{085AC320-CFBA-41C9-8F51-860055D28591}">
+          <x14:cfRule type="dataBar" id="{E1717276-8550-4700-8014-924D0A8786E3}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37707,7 +37707,7 @@
           <xm:sqref>I12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C9DF7F37-551B-4340-8CED-2F29928BBECE}">
+          <x14:cfRule type="dataBar" id="{E14950CF-8344-4F4B-983B-C53705049FF6}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -38049,7 +38049,7 @@
       <c r="Y8" s="9"/>
       <c r="Z8" s="9"/>
     </row>
-    <row r="9" spans="1:26">
+    <row r="9" spans="1:26" ht="27">
       <c r="A9" s="10" t="s">
         <v>139</v>
       </c>
@@ -43640,25 +43640,25 @@
         <v>80</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E4" s="10">
         <v>46298</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G4" s="10" t="s">
         <v>107</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
@@ -43684,13 +43684,13 @@
         <v>197</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E5" s="10">
         <v>46298</v>
@@ -43702,7 +43702,7 @@
         <v>108</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I5" s="9"/>
       <c r="J5" s="9"/>
@@ -43728,13 +43728,13 @@
         <v>199</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E6" s="10">
         <v>46298</v>
@@ -43746,7 +43746,7 @@
         <v>107</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I6" s="9"/>
       <c r="J6" s="9"/>
@@ -43775,10 +43775,10 @@
         <v>201</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E7" s="10">
         <v>46298</v>
@@ -43790,7 +43790,7 @@
         <v>107</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
@@ -43816,25 +43816,25 @@
         <v>84</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E8" s="10">
         <v>46298</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>107</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I8" s="9"/>
       <c r="J8" s="9"/>
@@ -43863,7 +43863,7 @@
         <v>203</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>204</v>
@@ -43878,7 +43878,7 @@
         <v>107</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="9"/>

</xml_diff>

<commit_message>
wording: calculated estimates instead of model labels; real keyword anchor from Google Ads; renamed data folders; rebuilt reports
</commit_message>
<xml_diff>
--- a/ЛР2-3_Объем_рынка/Excel/ЛР2-3_1_потенциальные_клиенты_TableMind.xlsx
+++ b/ЛР2-3_Объем_рынка/Excel/ЛР2-3_1_потенциальные_клиенты_TableMind.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-project-continuation-447426\ЛР2-3_Объем_рынка\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F6D6D31-175C-458B-B2AC-50134AF29623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFFBE24E-2FFB-4E1A-97C7-9AF623037A0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="458" windowWidth="12022" windowHeight="10972" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1165,7 +1165,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-9F8E-44C6-9199-F3F73541D651}"/>
+              <c16:uniqueId val="{00000000-1160-4222-BF93-5C64FBF6B95E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1231,7 +1231,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-9F8E-44C6-9199-F3F73541D651}"/>
+              <c16:uniqueId val="{00000001-1160-4222-BF93-5C64FBF6B95E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1397,7 +1397,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-93DF-4CA0-BFCA-F21826099D95}"/>
+              <c16:uniqueId val="{00000000-2792-4FCA-8913-71C0C44C0BDE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1445,7 +1445,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-93DF-4CA0-BFCA-F21826099D95}"/>
+              <c16:uniqueId val="{00000001-2792-4FCA-8913-71C0C44C0BDE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1493,7 +1493,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-93DF-4CA0-BFCA-F21826099D95}"/>
+              <c16:uniqueId val="{00000002-2792-4FCA-8913-71C0C44C0BDE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -37239,7 +37239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{19B092F5-97FB-4C0A-9C8C-40ABA9F679B2}</x14:id>
+          <x14:id>{CACD318B-223F-4524-BA86-690B9A61B19E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37253,7 +37253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BFED631D-F43A-4AB9-9CDC-C75D392666A3}</x14:id>
+          <x14:id>{40482C21-66C1-41F3-8DAC-4F699531526B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37285,7 +37285,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8CEF1969-B919-4D8A-B897-7D6D5A37F215}</x14:id>
+          <x14:id>{88C1BC73-0382-4A4F-842C-8EFD93759BDE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37299,7 +37299,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D7FF9E30-C39E-4C16-8821-6E9ADD4F048C}</x14:id>
+          <x14:id>{0D40575B-CFCA-4584-AB70-6B9DD796381F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37331,7 +37331,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{22A79C03-5308-48FD-92DE-AC368385D5F0}</x14:id>
+          <x14:id>{051EA58F-96DD-421F-9D93-4CFA746977BA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37345,7 +37345,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{78704DF2-01A5-4F19-9A2D-29E3748B20B2}</x14:id>
+          <x14:id>{A9A320CB-F557-44F0-B199-CB7856E06AAE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37377,7 +37377,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{25D83344-C72D-4CA8-B7C2-C73E123B3E99}</x14:id>
+          <x14:id>{2075BACD-E938-499C-B94D-DCC527CACECB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37391,7 +37391,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{868DCA10-951C-4065-961D-385D8E9AA796}</x14:id>
+          <x14:id>{5721D88D-650B-4EF6-8B05-55BBF1C0B261}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37423,7 +37423,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2CFC8904-BE06-4688-966A-50364C9C2093}</x14:id>
+          <x14:id>{EFD6820A-E476-4396-966E-86986665A1E9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37437,7 +37437,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{49EC93E7-804B-4E62-B374-28079E653682}</x14:id>
+          <x14:id>{8A4E42E6-8700-486B-A39C-43F05318AEAD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37469,7 +37469,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2ACA975A-79A2-477D-9FD8-A120D68F07C7}</x14:id>
+          <x14:id>{E72460FA-51B3-4A42-89DD-D1BDFD4511D9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37483,7 +37483,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{37699D38-4C97-4A44-8067-5EE2EC15DEC1}</x14:id>
+          <x14:id>{2AA2B836-5ABC-4F6E-A7D6-F76AB336D8D2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37515,7 +37515,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E1717276-8550-4700-8014-924D0A8786E3}</x14:id>
+          <x14:id>{F5044B8B-BAA2-4B04-ADDB-C89C2521348A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37529,7 +37529,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E14950CF-8344-4F4B-983B-C53705049FF6}</x14:id>
+          <x14:id>{0ACD48C1-E836-4446-9FD8-E499B8E4C580}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37564,7 +37564,7 @@
           <xm:sqref>O4:O5 O13:O15</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{19B092F5-97FB-4C0A-9C8C-40ABA9F679B2}">
+          <x14:cfRule type="dataBar" id="{CACD318B-223F-4524-BA86-690B9A61B19E}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37575,7 +37575,7 @@
           <xm:sqref>I6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BFED631D-F43A-4AB9-9CDC-C75D392666A3}">
+          <x14:cfRule type="dataBar" id="{40482C21-66C1-41F3-8DAC-4F699531526B}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37586,7 +37586,7 @@
           <xm:sqref>O6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8CEF1969-B919-4D8A-B897-7D6D5A37F215}">
+          <x14:cfRule type="dataBar" id="{88C1BC73-0382-4A4F-842C-8EFD93759BDE}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37597,7 +37597,7 @@
           <xm:sqref>I7</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D7FF9E30-C39E-4C16-8821-6E9ADD4F048C}">
+          <x14:cfRule type="dataBar" id="{0D40575B-CFCA-4584-AB70-6B9DD796381F}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37608,7 +37608,7 @@
           <xm:sqref>O7</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{22A79C03-5308-48FD-92DE-AC368385D5F0}">
+          <x14:cfRule type="dataBar" id="{051EA58F-96DD-421F-9D93-4CFA746977BA}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37619,7 +37619,7 @@
           <xm:sqref>I8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{78704DF2-01A5-4F19-9A2D-29E3748B20B2}">
+          <x14:cfRule type="dataBar" id="{A9A320CB-F557-44F0-B199-CB7856E06AAE}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37630,7 +37630,7 @@
           <xm:sqref>O8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{25D83344-C72D-4CA8-B7C2-C73E123B3E99}">
+          <x14:cfRule type="dataBar" id="{2075BACD-E938-499C-B94D-DCC527CACECB}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37641,7 +37641,7 @@
           <xm:sqref>I9</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{868DCA10-951C-4065-961D-385D8E9AA796}">
+          <x14:cfRule type="dataBar" id="{5721D88D-650B-4EF6-8B05-55BBF1C0B261}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37652,7 +37652,7 @@
           <xm:sqref>O9</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2CFC8904-BE06-4688-966A-50364C9C2093}">
+          <x14:cfRule type="dataBar" id="{EFD6820A-E476-4396-966E-86986665A1E9}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37663,7 +37663,7 @@
           <xm:sqref>I10</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{49EC93E7-804B-4E62-B374-28079E653682}">
+          <x14:cfRule type="dataBar" id="{8A4E42E6-8700-486B-A39C-43F05318AEAD}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37674,7 +37674,7 @@
           <xm:sqref>O10</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2ACA975A-79A2-477D-9FD8-A120D68F07C7}">
+          <x14:cfRule type="dataBar" id="{E72460FA-51B3-4A42-89DD-D1BDFD4511D9}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37685,7 +37685,7 @@
           <xm:sqref>I11</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{37699D38-4C97-4A44-8067-5EE2EC15DEC1}">
+          <x14:cfRule type="dataBar" id="{2AA2B836-5ABC-4F6E-A7D6-F76AB336D8D2}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37696,7 +37696,7 @@
           <xm:sqref>O11</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E1717276-8550-4700-8014-924D0A8786E3}">
+          <x14:cfRule type="dataBar" id="{F5044B8B-BAA2-4B04-ADDB-C89C2521348A}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -37707,7 +37707,7 @@
           <xm:sqref>I12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E14950CF-8344-4F4B-983B-C53705049FF6}">
+          <x14:cfRule type="dataBar" id="{0ACD48C1-E836-4446-9FD8-E499B8E4C580}">
             <x14:dataBar>
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>

</xml_diff>